<commit_message>
HP Bid (XLSX): qty from Min Order Qty; Max Deal Qty to Comments
For Part Number / Bundle lines, output Qty now derives from Min Order Qty
(0 -> 1) instead of Max Deal Qty. Max Deal Qty is written to the Comments
column as "Max Qty: {n}". Bundle Detail lines continue to take Qty from
Bundle Detail Qty and carry no Max Deal Qty, so their Comments stay blank.
Min Order Qty (col W) is unchanged.

Regenerated the four HP golden outputs and updated the parser tests and
docs (computed totals now 8314.59 and 34402.45 for the two samples).
</commit_message>
<xml_diff>
--- a/samples/outputs/Deals20260518T043243_HPI_NoCalculation_parsed.xlsx
+++ b/samples/outputs/Deals20260518T043243_HPI_NoCalculation_parsed.xlsx
@@ -114,6 +114,9 @@
     <x:t>HP USB-C Dock G5</x:t>
   </x:si>
   <x:si>
+    <x:t>Max Qty: 100</x:t>
+  </x:si>
+  <x:si>
     <x:t>2</x:t>
   </x:si>
   <x:si>
@@ -141,6 +144,9 @@
     <x:t>HP EB8G1I14 U5 225U 14 16GB/512 PC</x:t>
   </x:si>
   <x:si>
+    <x:t>Max Qty: 500</x:t>
+  </x:si>
+  <x:si>
     <x:t>5</x:t>
   </x:si>
   <x:si>
@@ -148,6 +154,9 @@
   </x:si>
   <x:si>
     <x:t>HP ZB8G1i14 U5 225H 14 16GB/512 PC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Max Qty: 250</x:t>
   </x:si>
   <x:si>
     <x:t>*</x:t>
@@ -613,10 +622,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I3" s="0">
         <x:v>165.83</x:v>
+      </x:c>
+      <x:c r="R3" s="0" t="s">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="W3" s="0">
         <x:v>1</x:v>
@@ -624,22 +636,25 @@
     </x:row>
     <x:row r="4" spans="1:27">
       <x:c r="A4" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="0">
         <x:v>336.7</x:v>
+      </x:c>
+      <x:c r="R4" s="0" t="s">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="W4" s="0">
         <x:v>1</x:v>
@@ -647,22 +662,25 @@
     </x:row>
     <x:row r="5" spans="1:27">
       <x:c r="A5" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>100</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="0">
         <x:v>3393.88</x:v>
+      </x:c>
+      <x:c r="R5" s="0" t="s">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="W5" s="0">
         <x:v>1</x:v>
@@ -670,22 +688,25 @@
     </x:row>
     <x:row r="6" spans="1:27">
       <x:c r="A6" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>500</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I6" s="0">
         <x:v>2258.18</x:v>
+      </x:c>
+      <x:c r="R6" s="0" t="s">
+        <x:v>42</x:v>
       </x:c>
       <x:c r="W6" s="0">
         <x:v>1</x:v>
@@ -693,22 +714,25 @@
     </x:row>
     <x:row r="7" spans="1:27">
       <x:c r="A7" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>250</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I7" s="0">
         <x:v>2160</x:v>
+      </x:c>
+      <x:c r="R7" s="0" t="s">
+        <x:v>46</x:v>
       </x:c>
       <x:c r="W7" s="0">
         <x:v>1</x:v>
@@ -716,10 +740,10 @@
     </x:row>
     <x:row r="8" spans="1:27">
       <x:c r="B8" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>